<commit_message>
feat: add program import feature with Excel and CSV templates, UI components, and tax store
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Arsip_Program_SCM.xlsx
+++ b/public/templates/Template_Import_Arsip_Program_SCM.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -411,6 +411,8 @@
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="24.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,6 +449,12 @@
       <c r="K1" t="str">
         <v>TOTAL INVOICE</v>
       </c>
+      <c r="L1" t="str">
+        <v>NO. FAKTUR PAJAK</v>
+      </c>
+      <c r="M1" t="str">
+        <v>TAX INVOICE DATE</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -482,6 +490,12 @@
       <c r="K2" s="1">
         <v>49950000</v>
       </c>
+      <c r="L2" t="str">
+        <v>010.002-26.11029381</v>
+      </c>
+      <c r="M2" t="str">
+        <v>2026-03-05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -517,6 +531,12 @@
       <c r="K3" s="1">
         <v>133200000</v>
       </c>
+      <c r="L3" t="str">
+        <v>010.002-26.22910382</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2026-03-08</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -552,6 +572,12 @@
       <c r="K4" s="1">
         <v>83250000</v>
       </c>
+      <c r="L4" t="str">
+        <v>010.002-26.33849102</v>
+      </c>
+      <c r="M4" t="str">
+        <v>2026-03-11</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -587,6 +613,12 @@
       <c r="K5" s="1">
         <v>42735000</v>
       </c>
+      <c r="L5" t="str">
+        <v>010.002-26.44910293</v>
+      </c>
+      <c r="M5" t="str">
+        <v>2026-03-14</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -622,6 +654,12 @@
       <c r="K6" s="1">
         <v>102120000</v>
       </c>
+      <c r="L6" t="str">
+        <v>010.002-26.55910294</v>
+      </c>
+      <c r="M6" t="str">
+        <v>2026-03-18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -657,6 +695,12 @@
       <c r="K7" s="1">
         <v>920000000</v>
       </c>
+      <c r="L7" t="str">
+        <v>010.002-26.66910295</v>
+      </c>
+      <c r="M7" t="str">
+        <v>2026-02-04</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -692,6 +736,12 @@
       <c r="K8" s="1">
         <v>1250000000</v>
       </c>
+      <c r="L8" t="str">
+        <v>010.002-26.77910296</v>
+      </c>
+      <c r="M8" t="str">
+        <v>2026-02-09</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -727,6 +777,12 @@
       <c r="K9" s="1">
         <v>720000000</v>
       </c>
+      <c r="L9" t="str">
+        <v>010.002-26.88910297</v>
+      </c>
+      <c r="M9" t="str">
+        <v>2026-02-15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -762,6 +818,12 @@
       <c r="K10" s="1">
         <v>550000000</v>
       </c>
+      <c r="L10" t="str">
+        <v>010.002-26.99910298</v>
+      </c>
+      <c r="M10" t="str">
+        <v>2026-02-20</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -797,6 +859,12 @@
       <c r="K11" s="1">
         <v>350000000</v>
       </c>
+      <c r="L11" t="str">
+        <v>010.002-26.10910299</v>
+      </c>
+      <c r="M11" t="str">
+        <v>2026-01-08</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -832,6 +900,12 @@
       <c r="K12" s="1">
         <v>180000000</v>
       </c>
+      <c r="L12" t="str">
+        <v>010.002-26.20910300</v>
+      </c>
+      <c r="M12" t="str">
+        <v>2026-01-14</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -867,10 +941,16 @@
       <c r="K13" s="1">
         <v>250000000</v>
       </c>
+      <c r="L13" t="str">
+        <v>010.002-26.30910301</v>
+      </c>
+      <c r="M13" t="str">
+        <v>2026-01-22</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement SCM program archive management module with UI components, backend API, and import templates
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Arsip_Program_SCM.xlsx
+++ b/public/templates/Template_Import_Arsip_Program_SCM.xlsx
@@ -11,7 +11,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="133">
+  <si>
+    <t>TANGGAL</t>
+  </si>
   <si>
     <t>BULAN</t>
   </si>
@@ -25,6 +28,9 @@
     <t>COMPANY NAME</t>
   </si>
   <si>
+    <t>KODE GUDANG</t>
+  </si>
+  <si>
     <t>NO. PO/SJ</t>
   </si>
   <si>
@@ -55,6 +61,9 @@
     <t>TAX INVOICE DATE</t>
   </si>
   <si>
+    <t>2026-03-05</t>
+  </si>
+  <si>
     <t>Maret 2026</t>
   </si>
   <si>
@@ -67,6 +76,9 @@
     <t>PT SCM Nusantara</t>
   </si>
   <si>
+    <t>GDG-JKT-01</t>
+  </si>
+  <si>
     <t>PO/2026/0101 / SJ-0101</t>
   </si>
   <si>
@@ -85,7 +97,7 @@
     <t>010.002-26.11029381</t>
   </si>
   <si>
-    <t>2026-03-05</t>
+    <t>2026-03-08</t>
   </si>
   <si>
     <t>Sewa Alat Berat</t>
@@ -97,6 +109,9 @@
     <t>PT SCM Solusi Indonesia</t>
   </si>
   <si>
+    <t>GDG-SBY-02</t>
+  </si>
+  <si>
     <t>PO/2026/0102 / SJ-0102</t>
   </si>
   <si>
@@ -115,7 +130,7 @@
     <t>010.002-26.22910382</t>
   </si>
   <si>
-    <t>2026-03-08</t>
+    <t>2026-03-11</t>
   </si>
   <si>
     <t>Inspeksi &amp; Sertifikasi</t>
@@ -124,6 +139,9 @@
     <t>Vidio</t>
   </si>
   <si>
+    <t>GDG-BDG-01</t>
+  </si>
+  <si>
     <t>PO/2026/0103 / SJ-0103</t>
   </si>
   <si>
@@ -142,7 +160,7 @@
     <t>010.002-26.33849102</t>
   </si>
   <si>
-    <t>2026-03-11</t>
+    <t>2026-03-14</t>
   </si>
   <si>
     <t>Mekanikal &amp; Valve</t>
@@ -154,6 +172,9 @@
     <t>PT SCM Logistik Utama</t>
   </si>
   <si>
+    <t>GDG-CKR-03</t>
+  </si>
+  <si>
     <t>PO/2026/0104 / SJ-0104</t>
   </si>
   <si>
@@ -172,7 +193,7 @@
     <t>010.002-26.44910293</t>
   </si>
   <si>
-    <t>2026-03-14</t>
+    <t>2026-03-18</t>
   </si>
   <si>
     <t>Bahan Kimia</t>
@@ -184,6 +205,9 @@
     <t>PT Surya Citra Media Tbk</t>
   </si>
   <si>
+    <t>GDG-TBN-01</t>
+  </si>
+  <si>
     <t>PO/2026/0105 / SJ-0105</t>
   </si>
   <si>
@@ -202,7 +226,7 @@
     <t>010.002-26.55910294</t>
   </si>
   <si>
-    <t>2026-03-18</t>
+    <t>2026-02-04</t>
   </si>
   <si>
     <t>Februari 2026</t>
@@ -214,6 +238,9 @@
     <t>SCM</t>
   </si>
   <si>
+    <t>GDG-JKT-02</t>
+  </si>
+  <si>
     <t>PO/2026/0201 / SJ-0201</t>
   </si>
   <si>
@@ -229,7 +256,7 @@
     <t>010.002-26.66910295</t>
   </si>
   <si>
-    <t>2026-02-04</t>
+    <t>2026-02-09</t>
   </si>
   <si>
     <t>IT &amp; Software</t>
@@ -250,12 +277,15 @@
     <t>010.002-26.77910296</t>
   </si>
   <si>
-    <t>2026-02-09</t>
+    <t>2026-02-15</t>
   </si>
   <si>
     <t>Distribusi</t>
   </si>
   <si>
+    <t>GDG-SMG-01</t>
+  </si>
+  <si>
     <t>PO/2026/0203 / SJ-0203</t>
   </si>
   <si>
@@ -271,12 +301,15 @@
     <t>010.002-26.88910297</t>
   </si>
   <si>
-    <t>2026-02-15</t>
+    <t>2026-02-20</t>
   </si>
   <si>
     <t>Material Handling</t>
   </si>
   <si>
+    <t>GDG-CKR-01</t>
+  </si>
+  <si>
     <t>PO/2026/0204 / SJ-0204</t>
   </si>
   <si>
@@ -295,7 +328,7 @@
     <t>010.002-26.99910298</t>
   </si>
   <si>
-    <t>2026-02-20</t>
+    <t>2026-01-08</t>
   </si>
   <si>
     <t>Januari 2026</t>
@@ -304,6 +337,9 @@
     <t>Warehouse</t>
   </si>
   <si>
+    <t>GDG-CKR-02</t>
+  </si>
+  <si>
     <t>PO/2026/0111 / SJ-0111</t>
   </si>
   <si>
@@ -322,12 +358,15 @@
     <t>010.002-26.10910299</t>
   </si>
   <si>
-    <t>2026-01-08</t>
+    <t>2026-01-14</t>
   </si>
   <si>
     <t>Packaging</t>
   </si>
   <si>
+    <t>GDG-SBY-01</t>
+  </si>
+  <si>
     <t>PO/2026/0112 / SJ-0112</t>
   </si>
   <si>
@@ -346,12 +385,15 @@
     <t>010.002-26.20910300</t>
   </si>
   <si>
-    <t>2026-01-14</t>
+    <t>2026-01-22</t>
   </si>
   <si>
     <t>Promosi</t>
   </si>
   <si>
+    <t>GDG-JKT-03</t>
+  </si>
+  <si>
     <t>PO/2026/0113 / SJ-0113</t>
   </si>
   <si>
@@ -368,9 +410,6 @@
   </si>
   <si>
     <t>010.002-26.30910301</t>
-  </si>
-  <si>
-    <t>2026-01-22</t>
   </si>
 </sst>
 </file>
@@ -836,25 +875,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="46" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="1" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="46" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="10" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -897,537 +937,615 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="4">
+        <v>45000000</v>
+      </c>
+      <c r="M2" s="4">
+        <v>4950000</v>
+      </c>
+      <c r="N2" s="5">
+        <v>49950000</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3" t="s">
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="C3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="8">
+        <v>120000000</v>
+      </c>
+      <c r="M3" s="8">
+        <v>13200000</v>
+      </c>
+      <c r="N3" s="9">
+        <v>133200000</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L4" s="4">
+        <v>75000000</v>
+      </c>
+      <c r="M4" s="4">
+        <v>8250000</v>
+      </c>
+      <c r="N4" s="5">
+        <v>83250000</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" s="8">
+        <v>38500000</v>
+      </c>
+      <c r="M5" s="8">
+        <v>4235000</v>
+      </c>
+      <c r="N5" s="9">
+        <v>42735000</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L6" s="4">
+        <v>92000000</v>
+      </c>
+      <c r="M6" s="4">
+        <v>10120000</v>
+      </c>
+      <c r="N6" s="5">
+        <v>102120000</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="L7" s="8">
+        <v>828828829</v>
+      </c>
+      <c r="M7" s="8">
+        <v>91171171</v>
+      </c>
+      <c r="N7" s="9">
+        <v>920000000</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L8" s="4">
+        <v>1126126126</v>
+      </c>
+      <c r="M8" s="4">
+        <v>123873874</v>
+      </c>
+      <c r="N8" s="5">
+        <v>1250000000</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="L9" s="8">
+        <v>648648649</v>
+      </c>
+      <c r="M9" s="8">
+        <v>71351351</v>
+      </c>
+      <c r="N9" s="9">
+        <v>720000000</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="E10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="L10" s="4">
+        <v>495495495</v>
+      </c>
+      <c r="M10" s="4">
+        <v>54504505</v>
+      </c>
+      <c r="N10" s="5">
+        <v>550000000</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="4">
-        <v>45000000</v>
-      </c>
-      <c r="K2" s="4">
-        <v>4950000</v>
-      </c>
-      <c r="L2" s="5">
-        <v>49950000</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>24</v>
+      <c r="F11" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="L11" s="8">
+        <v>315315315</v>
+      </c>
+      <c r="M11" s="8">
+        <v>34684685</v>
+      </c>
+      <c r="N11" s="9">
+        <v>350000000</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" s="6" t="s">
+    <row r="12" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" s="8">
-        <v>120000000</v>
-      </c>
-      <c r="K3" s="8">
-        <v>13200000</v>
-      </c>
-      <c r="L3" s="9">
-        <v>133200000</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>34</v>
+      <c r="F12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="L12" s="4">
+        <v>162162162</v>
+      </c>
+      <c r="M12" s="4">
+        <v>17837838</v>
+      </c>
+      <c r="N12" s="5">
+        <v>180000000</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="4">
-        <v>75000000</v>
-      </c>
-      <c r="K4" s="4">
-        <v>8250000</v>
-      </c>
-      <c r="L4" s="5">
-        <v>83250000</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="8">
-        <v>38500000</v>
-      </c>
-      <c r="K5" s="8">
-        <v>4235000</v>
-      </c>
-      <c r="L5" s="9">
-        <v>42735000</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J6" s="4">
-        <v>92000000</v>
-      </c>
-      <c r="K6" s="4">
-        <v>10120000</v>
-      </c>
-      <c r="L6" s="5">
-        <v>102120000</v>
-      </c>
-      <c r="M6" s="2" t="s">
+    <row r="13" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="E13" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="J7" s="8">
-        <v>828828829</v>
-      </c>
-      <c r="K7" s="8">
-        <v>91171171</v>
-      </c>
-      <c r="L7" s="9">
-        <v>920000000</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="J8" s="4">
-        <v>1126126126</v>
-      </c>
-      <c r="K8" s="4">
-        <v>123873874</v>
-      </c>
-      <c r="L8" s="5">
-        <v>1250000000</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J9" s="8">
-        <v>648648649</v>
-      </c>
-      <c r="K9" s="8">
-        <v>71351351</v>
-      </c>
-      <c r="L9" s="9">
-        <v>720000000</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="J10" s="4">
-        <v>495495495</v>
-      </c>
-      <c r="K10" s="4">
-        <v>54504505</v>
-      </c>
-      <c r="L10" s="5">
-        <v>550000000</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="J11" s="8">
-        <v>315315315</v>
-      </c>
-      <c r="K11" s="8">
-        <v>34684685</v>
-      </c>
-      <c r="L11" s="9">
-        <v>350000000</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J12" s="4">
-        <v>162162162</v>
-      </c>
-      <c r="K12" s="4">
-        <v>17837838</v>
-      </c>
-      <c r="L12" s="5">
-        <v>180000000</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="J13" s="8">
+      <c r="F13" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="L13" s="8">
         <v>225225225</v>
       </c>
-      <c r="K13" s="8">
+      <c r="M13" s="8">
         <v>24774775</v>
       </c>
-      <c r="L13" s="9">
+      <c r="N13" s="9">
         <v>250000000</v>
       </c>
-      <c r="M13" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>119</v>
+      <c r="O13" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement program import feature with excel modal, templates, and backend controller
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Arsip_Program_SCM.xlsx
+++ b/public/templates/Template_Import_Arsip_Program_SCM.xlsx
@@ -61,7 +61,7 @@
     <t>TAX INVOICE DATE</t>
   </si>
   <si>
-    <t>2026-03-05</t>
+    <t>05-03-2026</t>
   </si>
   <si>
     <t>Maret 2026</t>
@@ -97,7 +97,7 @@
     <t>010.002-26.11029381</t>
   </si>
   <si>
-    <t>2026-03-08</t>
+    <t>08-03-2026</t>
   </si>
   <si>
     <t>Sewa Alat Berat</t>
@@ -130,7 +130,7 @@
     <t>010.002-26.22910382</t>
   </si>
   <si>
-    <t>2026-03-11</t>
+    <t>11-03-2026</t>
   </si>
   <si>
     <t>Inspeksi &amp; Sertifikasi</t>
@@ -160,7 +160,7 @@
     <t>010.002-26.33849102</t>
   </si>
   <si>
-    <t>2026-03-14</t>
+    <t>14-03-2026</t>
   </si>
   <si>
     <t>Mekanikal &amp; Valve</t>
@@ -193,7 +193,7 @@
     <t>010.002-26.44910293</t>
   </si>
   <si>
-    <t>2026-03-18</t>
+    <t>18-03-2026</t>
   </si>
   <si>
     <t>Bahan Kimia</t>
@@ -226,7 +226,7 @@
     <t>010.002-26.55910294</t>
   </si>
   <si>
-    <t>2026-02-04</t>
+    <t>04-02-2026</t>
   </si>
   <si>
     <t>Februari 2026</t>
@@ -256,7 +256,7 @@
     <t>010.002-26.66910295</t>
   </si>
   <si>
-    <t>2026-02-09</t>
+    <t>09-02-2026</t>
   </si>
   <si>
     <t>IT &amp; Software</t>
@@ -277,7 +277,7 @@
     <t>010.002-26.77910296</t>
   </si>
   <si>
-    <t>2026-02-15</t>
+    <t>15-02-2026</t>
   </si>
   <si>
     <t>Distribusi</t>
@@ -301,7 +301,7 @@
     <t>010.002-26.88910297</t>
   </si>
   <si>
-    <t>2026-02-20</t>
+    <t>20-02-2026</t>
   </si>
   <si>
     <t>Material Handling</t>
@@ -328,7 +328,7 @@
     <t>010.002-26.99910298</t>
   </si>
   <si>
-    <t>2026-01-08</t>
+    <t>08-01-2026</t>
   </si>
   <si>
     <t>Januari 2026</t>
@@ -358,7 +358,7 @@
     <t>010.002-26.10910299</t>
   </si>
   <si>
-    <t>2026-01-14</t>
+    <t>14-01-2026</t>
   </si>
   <si>
     <t>Packaging</t>
@@ -385,7 +385,7 @@
     <t>010.002-26.20910300</t>
   </si>
   <si>
-    <t>2026-01-22</t>
+    <t>22-01-2026</t>
   </si>
   <si>
     <t>Promosi</t>
@@ -507,9 +507,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -523,6 +526,9 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -948,46 +954,46 @@
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="5">
         <v>45000000</v>
       </c>
-      <c r="M2" s="4">
+      <c r="M2" s="5">
         <v>4950000</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="6">
         <v>49950000</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="2" t="s">
@@ -995,52 +1001,52 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="10">
         <v>120000000</v>
       </c>
-      <c r="M3" s="8">
+      <c r="M3" s="10">
         <v>13200000</v>
       </c>
-      <c r="N3" s="9">
+      <c r="N3" s="11">
         <v>133200000</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="7" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1048,46 +1054,46 @@
       <c r="A4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="5">
         <v>75000000</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="5">
         <v>8250000</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>83250000</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="3" t="s">
         <v>48</v>
       </c>
       <c r="P4" s="2" t="s">
@@ -1095,52 +1101,52 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="10">
         <v>38500000</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="10">
         <v>4235000</v>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="11">
         <v>42735000</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="P5" s="6" t="s">
+      <c r="P5" s="7" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1148,46 +1154,46 @@
       <c r="A6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="5">
         <v>92000000</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>10120000</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="6">
         <v>102120000</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="3" t="s">
         <v>70</v>
       </c>
       <c r="P6" s="2" t="s">
@@ -1195,52 +1201,52 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="10">
         <v>828828829</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="10">
         <v>91171171</v>
       </c>
-      <c r="N7" s="9">
+      <c r="N7" s="11">
         <v>920000000</v>
       </c>
-      <c r="O7" s="6" t="s">
+      <c r="O7" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="P7" s="7" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1248,46 +1254,46 @@
       <c r="A8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="5">
         <v>1126126126</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="5">
         <v>123873874</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="6">
         <v>1250000000</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="O8" s="3" t="s">
         <v>87</v>
       </c>
       <c r="P8" s="2" t="s">
@@ -1295,52 +1301,52 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="10">
         <v>648648649</v>
       </c>
-      <c r="M9" s="8">
+      <c r="M9" s="10">
         <v>71351351</v>
       </c>
-      <c r="N9" s="9">
+      <c r="N9" s="11">
         <v>720000000</v>
       </c>
-      <c r="O9" s="6" t="s">
+      <c r="O9" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="P9" s="6" t="s">
+      <c r="P9" s="7" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1348,46 +1354,46 @@
       <c r="A10" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="5">
         <v>495495495</v>
       </c>
-      <c r="M10" s="4">
+      <c r="M10" s="5">
         <v>54504505</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="6">
         <v>550000000</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="3" t="s">
         <v>104</v>
       </c>
       <c r="P10" s="2" t="s">
@@ -1395,52 +1401,52 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="K11" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="10">
         <v>315315315</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="10">
         <v>34684685</v>
       </c>
-      <c r="N11" s="9">
+      <c r="N11" s="11">
         <v>350000000</v>
       </c>
-      <c r="O11" s="6" t="s">
+      <c r="O11" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="P11" s="6" t="s">
+      <c r="P11" s="7" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1448,46 +1454,46 @@
       <c r="A12" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="5">
         <v>162162162</v>
       </c>
-      <c r="M12" s="4">
+      <c r="M12" s="5">
         <v>17837838</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="6">
         <v>180000000</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="O12" s="3" t="s">
         <v>123</v>
       </c>
       <c r="P12" s="2" t="s">
@@ -1495,52 +1501,52 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="L13" s="8">
+      <c r="L13" s="10">
         <v>225225225</v>
       </c>
-      <c r="M13" s="8">
+      <c r="M13" s="10">
         <v>24774775</v>
       </c>
-      <c r="N13" s="9">
+      <c r="N13" s="11">
         <v>250000000</v>
       </c>
-      <c r="O13" s="6" t="s">
+      <c r="O13" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="P13" s="6" t="s">
+      <c r="P13" s="7" t="s">
         <v>124</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement program management module with AI document analysis, payment status tracking, and Vue frontend views
</commit_message>
<xml_diff>
--- a/public/templates/Template_Import_Arsip_Program_SCM.xlsx
+++ b/public/templates/Template_Import_Arsip_Program_SCM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="120">
   <si>
     <t>TANGGAL</t>
   </si>
@@ -55,6 +55,9 @@
     <t>TOTAL INVOICE</t>
   </si>
   <si>
+    <t>STATUS PAYMENT</t>
+  </si>
+  <si>
     <t>NO. FAKTUR PAJAK</t>
   </si>
   <si>
@@ -94,6 +97,9 @@
     <t>INV/2026/SCM/0101</t>
   </si>
   <si>
+    <t>PAID</t>
+  </si>
+  <si>
     <t>010.002-26.11029381</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>INV/2026/SCM/0102</t>
   </si>
   <si>
+    <t>tempo</t>
+  </si>
+  <si>
     <t>010.002-26.22910382</t>
   </si>
   <si>
@@ -157,6 +166,9 @@
     <t>INV/2026/SCM/0103</t>
   </si>
   <si>
+    <t>WAITING PAYMENT</t>
+  </si>
+  <si>
     <t>010.002-26.33849102</t>
   </si>
   <si>
@@ -190,6 +202,9 @@
     <t>INV/2026/SCM/0104</t>
   </si>
   <si>
+    <t>cbd</t>
+  </si>
+  <si>
     <t>010.002-26.44910293</t>
   </si>
   <si>
@@ -356,60 +371,6 @@
   </si>
   <si>
     <t>010.002-26.10910299</t>
-  </si>
-  <si>
-    <t>14-01-2026</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-  </si>
-  <si>
-    <t>GDG-SBY-01</t>
-  </si>
-  <si>
-    <t>PO/2026/0112 / SJ-0112</t>
-  </si>
-  <si>
-    <t>Pengadaan Kemasan Corrugated Box &amp; Stretch Film</t>
-  </si>
-  <si>
-    <t>PT Riau Sakti Packaging Industries</t>
-  </si>
-  <si>
-    <t>01.884.223.5-021.000</t>
-  </si>
-  <si>
-    <t>INV/RSP/2026/0991</t>
-  </si>
-  <si>
-    <t>010.002-26.20910300</t>
-  </si>
-  <si>
-    <t>22-01-2026</t>
-  </si>
-  <si>
-    <t>Promosi</t>
-  </si>
-  <si>
-    <t>GDG-JKT-03</t>
-  </si>
-  <si>
-    <t>PO/2026/0113 / SJ-0113</t>
-  </si>
-  <si>
-    <t>Pengadaan Booth Branding &amp; Material Event SCM Expo</t>
-  </si>
-  <si>
-    <t>PT Mahaka Visual Integrasi</t>
-  </si>
-  <si>
-    <t>03.119.445.6-072.000</t>
-  </si>
-  <si>
-    <t>INV/MVI/2026/0219</t>
-  </si>
-  <si>
-    <t>010.002-26.30910301</t>
   </si>
 </sst>
 </file>
@@ -881,7 +842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -896,11 +857,12 @@
     <col min="12" max="12" width="20" customWidth="1"/>
     <col min="13" max="13" width="18" customWidth="1"/>
     <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="24" customWidth="1"/>
-    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -949,40 +911,43 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L2" s="5">
         <v>45000000</v>
@@ -994,45 +959,48 @@
         <v>49950000</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>16</v>
+        <v>28</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L3" s="10">
         <v>120000000</v>
@@ -1044,45 +1012,48 @@
         <v>133200000</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>28</v>
+        <v>40</v>
+      </c>
+      <c r="P3" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="L4" s="5">
         <v>75000000</v>
@@ -1094,45 +1065,48 @@
         <v>83250000</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>39</v>
+        <v>51</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="L5" s="10">
         <v>38500000</v>
@@ -1144,45 +1118,48 @@
         <v>42735000</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>49</v>
+        <v>63</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L6" s="5">
         <v>92000000</v>
@@ -1194,45 +1171,48 @@
         <v>102120000</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>60</v>
+        <v>28</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="L7" s="10">
         <v>828828829</v>
@@ -1244,45 +1224,48 @@
         <v>920000000</v>
       </c>
       <c r="O7" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>71</v>
+        <v>40</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>76</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L8" s="5">
         <v>1126126126</v>
@@ -1294,45 +1277,48 @@
         <v>1250000000</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>81</v>
+        <v>51</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L9" s="10">
         <v>648648649</v>
@@ -1344,45 +1330,48 @@
         <v>720000000</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>88</v>
+        <v>28</v>
+      </c>
+      <c r="P9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>93</v>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="L10" s="5">
         <v>495495495</v>
@@ -1394,45 +1383,48 @@
         <v>550000000</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="P10" s="2" t="s">
-        <v>96</v>
+        <v>63</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" ht="22" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="L11" s="10">
         <v>315315315</v>
@@ -1444,114 +1436,17 @@
         <v>350000000</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="P11" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="H12" s="4" t="s">
+      <c r="P11" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="I12" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="L12" s="5">
-        <v>162162162</v>
-      </c>
-      <c r="M12" s="5">
-        <v>17837838</v>
-      </c>
-      <c r="N12" s="6">
-        <v>180000000</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="P12" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="L13" s="10">
-        <v>225225225</v>
-      </c>
-      <c r="M13" s="10">
-        <v>24774775</v>
-      </c>
-      <c r="N13" s="11">
-        <v>250000000</v>
-      </c>
-      <c r="O13" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="P13" s="7" t="s">
-        <v>124</v>
+      <c r="Q11" s="7" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>